<commit_message>
Add the PDF audit report promised in Review 1
08_Report_PDF renders a formal, print-styled audit document and prints it to
PDF with headless Edge (Chrome as fallback). No PDF library and no Office
dependency, so it behaves identically on an unattended robot. Unlike the
dashboard it lists every transaction, records a SHA-256 of Config.xlsx so the
exact configuration used is pinned, and closes with the audit chain head.

A missing browser degrades to the HTML copy with a warning rather than failing
the run, since the audit log rather than this document is the record.

Also fixes settings drift in the data generator: six settings had been added
straight to Config.xlsx and would have been silently dropped by a regenerate.
The generator is the single source of truth again. ExplorerAddressUrl, which
nothing read, is removed.
</commit_message>
<xml_diff>
--- a/BlockchainLogisticsValidator/Data/Config.xlsx
+++ b/BlockchainLogisticsValidator/Data/Config.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -547,6 +547,7 @@
           <t>EtherscanApiKey</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Free key from etherscan.io/myapikey. Blank keeps API mode disabled.</t>
@@ -588,17 +589,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ExplorerAddressUrl</t>
+          <t>ExplorerPageUrl</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://etherscan.io/address/{0}</t>
+          <t>Data\Input\MockChain\explorer_ethereum.html</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Used when DataSourceMode = WEB.</t>
+          <t>Used when DataSourceMode = WEB. A project-relative page, or a live explorer URL.</t>
         </is>
       </c>
     </row>
@@ -620,462 +621,483 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LogisticsFile</t>
+          <t>RunMode</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Data\Input\LogisticsRecords.xlsx</t>
+          <t>BATCH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ERP / WMS export.</t>
+          <t>BATCH validates the whole run in one job; DISPATCH splits it into one Orchestrator queue item per shipment.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ShipmentsSheet</t>
+          <t>QueueMode</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Shipments</t>
+          <t>DRYRUN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Shipment master sheet name.</t>
+          <t>ORCHESTRATOR pushes real queue items; DRYRUN writes the payloads to disk for inspection.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ShipmentEventsSheet</t>
+          <t>QueueName</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ShipmentEvents</t>
+          <t>BlockchainValidationQueue</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Expected milestone lines.</t>
+          <t>Orchestrator queue used by Dispatcher and Performer.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TxShipmentMapFile</t>
+          <t>LogisticsFile</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Data\Input\TxShipmentMap.xlsx</t>
+          <t>Data\Input\LogisticsRecords.xlsx</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Used when MappingMode = LOOKUP.</t>
+          <t>ERP / WMS export.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MappingMode</t>
+          <t>ShipmentsSheet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DECODE</t>
+          <t>Shipments</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DECODE reads the ABI input data; LOOKUP uses the mapping file.</t>
+          <t>Shipment master sheet name.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TimestampToleranceHours</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
+          <t>ShipmentEventsSheet</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ShipmentEvents</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>R1: drift up to this is a PASS.</t>
+          <t>Expected milestone lines.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TimestampWarnToleranceHours</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>4</v>
+          <t>TxShipmentMapFile</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Data\Input\TxShipmentMap.xlsx</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>R1: drift past this is a FAIL; between the two is a WARNING.</t>
+          <t>Used when MappingMode = LOOKUP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>QuantityTolerance</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0</v>
+          <t>MappingMode</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DECODE</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>R2: permitted absolute difference in units.</t>
+          <t>DECODE reads the ABI input data; LOOKUP uses the mapping file.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EscalationEnabled</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+          <t>TimestampToleranceHours</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Novelty 2: show the review form on a CRITICAL anomaly.</t>
+          <t>R1: drift up to this is a PASS.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>EscalationSeverity</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
+          <t>TimestampWarnToleranceHours</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Minimum severity that pauses the bot for a human.</t>
+          <t>R1: drift past this is a FAIL; between the two is a WARNING.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AttendedMode</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+          <t>QuantityTolerance</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>False in unattended runs: log and continue instead of blocking.</t>
+          <t>R2: permitted absolute difference in units.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AlertMode</t>
+          <t>EscalationEnabled</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EML</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EML writes the message to disk; SMTP and OUTLOOK actually send.</t>
+          <t>Novelty 2: show the review form on a CRITICAL anomaly.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AlertFrom</t>
+          <t>EscalationSeverity</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>rpa.bot@logistics-demo.local</t>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Minimum severity that pauses the bot for a human.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AlertTo</t>
+          <t>AttendedMode</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>logistics.manager@logistics-demo.local;compliance@logistics-demo.local</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Semicolon separated.</t>
+          <t>False in unattended runs: log and continue instead of blocking.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SmtpHost</t>
+          <t>EscalationMode</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>smtp.gmail.com</t>
+          <t>SIMULATE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Only used when AlertMode = SMTP.</t>
+          <t>PROMPT shows a reviewer dialog (attended only); SIMULATE applies the decision below; AUTO_LOG defers.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SmtpPort</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>587</v>
+          <t>SimulatedEscalationDecision</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>REJECTED - hold the shipment and open an investigation</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Used when EscalationMode = SIMULATE, so rehearsals produce the same artefacts as a real review.</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SmtpUseSsl</t>
+          <t>AlertMode</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>EML</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EML writes the message to disk; SMTP and OUTLOOK actually send.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SmtpUser</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Leave blank unless AlertMode = SMTP.</t>
-        </is>
-      </c>
+          <t>AlertFrom</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>rpa.bot@logistics-demo.local</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SmtpPassword</t>
+          <t>AlertTo</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>logistics.manager@logistics-demo.local;compliance@logistics-demo.local</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>App password. Never commit a real value.</t>
+          <t>Semicolon separated.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ReportsFolder</t>
+          <t>SmtpHost</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Data\Output\Reports</t>
+          <t>smtp.gmail.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Only used when AlertMode = SMTP.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AuditLogFolder</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Data\Output\AuditLogs</t>
-        </is>
-      </c>
+          <t>SmtpPort</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>587</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AuditLogFile</t>
+          <t>SmtpUseSsl</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ValidationAuditLog.csv</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Append-only, hash-chained.</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ScreenshotFolder</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Data\Output\Screenshots</t>
+          <t>SmtpUser</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Leave blank unless AlertMode = SMTP.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LogLevel</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Info</t>
-        </is>
-      </c>
+          <t>SmtpPassword</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Info | Trace.</t>
+          <t>App password. Never commit a real value.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>EscalationMode</t>
+          <t>ReportsFolder</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SIMULATE</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>PROMPT shows a reviewer dialog (attended only); SIMULATE applies the decision below; AUTO_LOG defers.</t>
-        </is>
-      </c>
+          <t>Data\Output\Reports</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SimulatedEscalationDecision</t>
+          <t>AuditLogFolder</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>REJECTED - hold the shipment and open an investigation</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Used when EscalationMode = SIMULATE, so rehearsals produce the same artefacts as a real review.</t>
-        </is>
-      </c>
+          <t>Data\Output\AuditLogs</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>QueueMode</t>
+          <t>AuditLogFile</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DRYRUN</t>
+          <t>ValidationAuditLog.csv</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ORCHESTRATOR pushes real queue items; DRYRUN writes the payloads to disk for inspection.</t>
+          <t>Append-only, hash-chained.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>QueueName</t>
+          <t>ScreenshotFolder</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BlockchainValidationQueue</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Orchestrator queue used by Dispatcher and Performer.</t>
-        </is>
-      </c>
+          <t>Data\Output\Screenshots</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RunMode</t>
+          <t>PdfReportEnabled</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BATCH</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BATCH validates the whole run in one job; DISPATCH splits it into one Orchestrator queue item per shipment.</t>
+          <t>Print the formal audit report to PDF with headless Edge.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ExplorerPageUrl</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Data\Input\MockChain\explorer_ethereum.html</t>
-        </is>
-      </c>
+          <t>PdfBrowserPath</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Used when DataSourceMode = WEB. A local replica by default; point at a live explorer URL and re-record the selector to scrape the real thing.</t>
+          <t>Blank finds Edge or Chrome automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LogLevel</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Info | Trace.</t>
         </is>
       </c>
     </row>
@@ -1207,6 +1229,7 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1239,6 +1262,8 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>ESCALATE</t>
@@ -1271,6 +1296,8 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1303,6 +1330,8 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1340,6 +1369,7 @@
           <t>GoodsReceived</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1605,6 +1635,7 @@
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1666,6 +1697,7 @@
           <t>LOWERCASE</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
Run in UiPath Studio only: remove every Orchestrator dependency
The project no longer touches Orchestrator. Dispatcher and Performer keep the
per-shipment split, but the queue is now a local work-queue file under
Reports\WorkQueue: Add Queue Item, Get Transaction Item and Set Transaction
Status are gone, as are the QueueMode and QueueName settings. QueueDryRunFile
becomes QueueFile. The Performer is still its own entry point, run from Studio.

The Orchestrator runbook is deleted. The README, user guide, traceability
matrix, results, demo script, speaking notes, checklist and deck generator now
say plainly that Orchestrator is out of scope and how queue mode works instead.

Verified: 57/57 Invoke Code bodies compile; dispatch writes 12 work items and
the Performer processes them to total=48 pass=40 warn=1 fail=7 escalations=1
with a VALID audit chain.
</commit_message>
<xml_diff>
--- a/BlockchainLogisticsValidator/Data/Config.xlsx
+++ b/BlockchainLogisticsValidator/Data/Config.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,7 @@
           <t>EtherscanApiKey</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Free key from etherscan.io/myapikey. Blank keeps API mode disabled.</t>
@@ -905,6 +906,7 @@
           <t>SmtpUser</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Leave blank for an unauthenticated relay.</t>
@@ -917,6 +919,7 @@
           <t>SmtpPassword</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>App password. Never commit a real value - use Config.local.json.</t>
@@ -1045,381 +1048,352 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>QueueMode</t>
+          <t>RunMode</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DRYRUN</t>
+          <t>BATCH</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ORCHESTRATOR pushes real queue items; DRYRUN writes the payloads to disk for inspection.</t>
+          <t>BATCH validates the whole run in one job; DISPATCH writes a work queue file, one item per shipment, for Workflows\Queue\Performer.xaml to process.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>QueueName</t>
+          <t>ExplorerPageUrl</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BlockchainValidationQueue</t>
+          <t>Data\Input\MockChain\explorer_ethereum.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Orchestrator queue used by Dispatcher and Performer.</t>
+          <t>Used when DataSourceMode = WEB. A local replica by default; point at a live explorer URL to scrape the real thing.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RunMode</t>
+          <t>ChainRecordsPath</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BATCH</t>
+          <t>result</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BATCH validates the whole run in one job; DISPATCH splits it into one Orchestrator queue item per shipment.</t>
+          <t>JSON path of the transaction array in a MOCK/API response. 'result' for Etherscan.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ExplorerPageUrl</t>
+          <t>FieldMappingSheet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Data\Input\MockChain\explorer_ethereum.html</t>
+          <t>FieldMapping</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Used when DataSourceMode = WEB. A local replica by default; point at a live explorer URL to scrape the real thing.</t>
+          <t>Which mapping sheet translates the feed's fields. FieldMapping = Etherscan; FieldMapping_EvmEtl = ethereum-etl export.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ChainRecordsPath</t>
+          <t>LogisticsSourceMode</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>EXCEL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JSON path of the transaction array in a MOCK/API response. 'result' for Etherscan.</t>
+          <t>EXCEL | CSV | SQL - where the ERP/WMS records are read from.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FieldMappingSheet</t>
+          <t>ShipmentsCsvFile</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FieldMapping</t>
+          <t>Data\Input\ERP_CSV\Shipments.csv</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Which mapping sheet translates the feed's fields. FieldMapping = Etherscan; FieldMapping_EvmEtl = ethereum-etl export.</t>
+          <t>Used when LogisticsSourceMode = CSV.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LogisticsSourceMode</t>
+          <t>ShipmentEventsCsvFile</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EXCEL</t>
+          <t>Data\Input\ERP_CSV\ShipmentEvents.csv</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>EXCEL | CSV | SQL - where the ERP/WMS records are read from.</t>
+          <t>Used when LogisticsSourceMode = CSV.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ShipmentsCsvFile</t>
+          <t>DbProviderName</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Data\Input\ERP_CSV\Shipments.csv</t>
+          <t>System.Data.Odbc</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Used when LogisticsSourceMode = CSV.</t>
+          <t>SQL mode: ADO.NET provider for Database Connect (System.Data.Odbc, System.Data.SqlClient, ...).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ShipmentEventsCsvFile</t>
+          <t>DbConnectionString</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Data\Input\ERP_CSV\ShipmentEvents.csv</t>
+          <t>Driver={Microsoft Access Driver (*.mdb, *.accdb)};Dbq={ProjectRoot}\Data\Input\LogisticsERP.accdb;</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Used when LogisticsSourceMode = CSV.</t>
+          <t>SQL mode. {ProjectRoot} is replaced at run time. Put real credentials in Config.local.json.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DbProviderName</t>
+          <t>DbShipmentsQuery</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>System.Data.Odbc</t>
+          <t>SELECT * FROM Shipments ORDER BY ShipmentID</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SQL mode: ADO.NET provider for Database Connect (System.Data.Odbc, System.Data.SqlClient, ...).</t>
+          <t>SQL mode: must return the Shipments columns.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DbConnectionString</t>
+          <t>DbShipmentEventsQuery</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Driver={Microsoft Access Driver (*.mdb, *.accdb)};Dbq={ProjectRoot}\Data\Input\LogisticsERP.accdb;</t>
+          <t>SELECT * FROM ShipmentEvents ORDER BY ShipmentID, ExpectedEventTimestampUtc</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SQL mode. {ProjectRoot} is replaced at run time. Put real credentials in Config.local.json.</t>
+          <t>SQL mode: must return the ShipmentEvents columns.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DbShipmentsQuery</t>
+          <t>ReviewUi</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SELECT * FROM Shipments ORDER BY ShipmentID</t>
+          <t>WINDOW</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SQL mode: must return the Shipments columns.</t>
+          <t>PROMPT mode: WINDOW shows the full review form; DIALOG falls back to a simple Input Dialog.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DbShipmentEventsQuery</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>SELECT * FROM ShipmentEvents ORDER BY ShipmentID, ExpectedEventTimestampUtc</t>
-        </is>
+          <t>ReviewTimeoutMinutes</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>30</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SQL mode: must return the ShipmentEvents columns.</t>
+          <t>An unanswered review window closes after this long and the item is recorded as DEFERRED.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ReviewUi</t>
+          <t>AlertAttachReports</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>WINDOW</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PROMPT mode: WINDOW shows the full review form; DIALOG falls back to a simple Input Dialog.</t>
+          <t>Attach the Excel and PDF reports to SMTP / Outlook alerts.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ReviewTimeoutMinutes</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>30</v>
-      </c>
+          <t>OutlookAccount</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>An unanswered review window closes after this long and the item is recorded as DEFERRED.</t>
+          <t>OUTLOOK mode: send from this account. Blank = the default profile.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AlertAttachReports</t>
+          <t>OutlookSaveAsDraft</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Attach the Excel and PDF reports to SMTP / Outlook alerts.</t>
+          <t>OUTLOOK mode: True saves the alert as a draft instead of sending it.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OutlookAccount</t>
-        </is>
-      </c>
+          <t>TeamsWebhookUrl</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>OUTLOOK mode: send from this account. Blank = the default profile.</t>
+          <t>Teams Workflows webhook. Blank writes the Adaptive Card payload to Reports instead of posting.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OutlookSaveAsDraft</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
+          <t>SlackWebhookUrl</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OUTLOOK mode: True saves the alert as a draft instead of sending it.</t>
+          <t>Slack incoming webhook. Blank writes the payload to Reports instead of posting.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TeamsWebhookUrl</t>
-        </is>
-      </c>
+          <t>DashboardPushUrl</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Teams Workflows webhook. Blank writes the Adaptive Card payload to Reports instead of posting.</t>
+          <t>Optional: Power BI streaming-dataset push URL or a Google Apps Script web app. Blank = no push.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SlackWebhookUrl</t>
+          <t>DashboardPushFormat</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>POWERBI</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Slack incoming webhook. Blank writes the payload to Reports instead of posting.</t>
+          <t>POWERBI posts one flat KPI row; JSON posts the full dashboard_summary.json document.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DashboardPushUrl</t>
+          <t>RunHistoryFile</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>RunHistory.csv</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Optional: Power BI streaming-dataset push URL or a Google Apps Script web app. Blank = no push.</t>
+          <t>Per-run KPIs and processing time, kept beside the audit log for trend charts.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DashboardPushFormat</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>POWERBI</t>
-        </is>
-      </c>
+          <t>QueueFile</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>POWERBI posts one flat KPI row; JSON posts the full dashboard_summary.json document.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>RunHistoryFile</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>RunHistory.csv</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Per-run KPIs and processing time, kept beside the audit log for trend charts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>QueueDryRunFile</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Performer in DRYRUN mode: payload file to process. Blank = the newest file in Reports\QueueDryRun.</t>
+          <t>Performer: work queue file to process. Blank = the newest file in Reports\WorkQueue.</t>
         </is>
       </c>
     </row>
@@ -1551,6 +1525,7 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1583,6 +1558,8 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>ESCALATE</t>
@@ -1615,6 +1592,8 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1647,6 +1626,8 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1684,6 +1665,7 @@
           <t>GoodsReceived</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>FLAG</t>
@@ -1949,6 +1931,7 @@
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2010,6 +1993,7 @@
           <t>LOWERCASE</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2223,6 +2207,7 @@
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2262,6 +2247,7 @@
           <t>LOWERCASE</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2279,6 +2265,7 @@
           <t>LOWERCASE</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2318,6 +2305,7 @@
           <t>ABI_STRING</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2335,6 +2323,7 @@
           <t>ABI_UINT256</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2352,6 +2341,7 @@
           <t>ABI_STRING</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2391,6 +2381,7 @@
           <t>LOWERCASE</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>